<commit_message>
feat(planet): derive permanent luck from reforge rewards
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/planet_buff.xlsx
+++ b/space-battleship/config_excel/planet_buff.xlsx
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K38"/>
+  <dimension ref="A1:K44"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.39999961853027"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="10"/>
@@ -2877,6 +2877,288 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>36</v>
+      </c>
+      <c r="B39" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="H39" t="n">
+        <v>100</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>7</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>永久幸运 +{value}</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>37</v>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="H40" t="n">
+        <v>100</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>7</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>永久幸运 +{value}</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>38</v>
+      </c>
+      <c r="B41" t="n">
+        <v>3</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>0</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="H41" t="n">
+        <v>100</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>7</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>永久幸运 +{value}</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>39</v>
+      </c>
+      <c r="B42" t="n">
+        <v>4</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="H42" t="n">
+        <v>100</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>7</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>永久幸运 +{value}</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>40</v>
+      </c>
+      <c r="B43" t="n">
+        <v>5</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="H43" t="n">
+        <v>100</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>7</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>永久幸运 +{value}</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>41</v>
+      </c>
+      <c r="B44" t="n">
+        <v>6</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>luck</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>all</t>
+        </is>
+      </c>
+      <c r="H44" t="n">
+        <v>100</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>7</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>永久幸运 +{value}</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Remove planetary hightech level rewards and refresh reward tests
</commit_message>
<xml_diff>
--- a/space-battleship/config_excel/planet_buff.xlsx
+++ b/space-battleship/config_excel/planet_buff.xlsx
@@ -1054,7 +1054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K44"/>
+  <dimension ref="A1:K38"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9" defaultRowHeight="14.39999961853027"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="10"/>
@@ -1281,7 +1281,7 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B5" t="n">
         <v>1</v>
@@ -1301,16 +1301,16 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>free_charge</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>hightech</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H5" t="n">
-        <v>25</v>
+        <v>0.1</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
@@ -1318,17 +1318,17 @@
         </is>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>AI工厂效果等级 +25</t>
+          <t>所有充能模块免费充能 +10%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B6" t="n">
         <v>1</v>
@@ -1348,16 +1348,16 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>free_charge</t>
+          <t>level_bonus</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>enhancement</t>
         </is>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
@@ -1365,17 +1365,17 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>所有充能模块免费充能 +10%</t>
+          <t>强化附加等级 +1</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B7" t="n">
         <v>1</v>
@@ -1395,12 +1395,12 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>crew_exp_share</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -1408,24 +1408,24 @@
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>add</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>强化附加等级 +1</t>
+          <t>本星球探索经验同步至所有船员</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -1469,10 +1469,10 @@
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -1516,10 +1516,10 @@
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -1563,10 +1563,10 @@
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -1610,10 +1610,10 @@
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -1657,10 +1657,10 @@
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B13" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -1677,34 +1677,34 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>crew_exp_share</t>
+          <t>level_bonus</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>equipment</t>
         </is>
       </c>
       <c r="H13" t="n">
+        <v>15</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
         <v>1</v>
       </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>max</t>
-        </is>
-      </c>
-      <c r="J13" t="n">
-        <v>5</v>
-      </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>本星球探索经验同步至所有船员</t>
+          <t>装备效果等级 +15</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B14" t="n">
         <v>2</v>
@@ -1724,16 +1724,16 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>free_charge</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>equipment</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H14" t="n">
-        <v>15</v>
+        <v>0.1</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -1741,17 +1741,17 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>装备效果等级 +15</t>
+          <t>所有充能模块免费充能 +10%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B15" t="n">
         <v>2</v>
@@ -1776,11 +1776,11 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>hightech</t>
+          <t>enhancement</t>
         </is>
       </c>
       <c r="H15" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1788,20 +1788,20 @@
         </is>
       </c>
       <c r="J15" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>AI工厂效果等级 +10</t>
+          <t>强化附加等级 +1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B16" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1818,16 +1818,16 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>free_charge</t>
+          <t>level_bonus</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>equipment</t>
         </is>
       </c>
       <c r="H16" t="n">
-        <v>0.1</v>
+        <v>15</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1835,20 +1835,20 @@
         </is>
       </c>
       <c r="J16" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>所有充能模块免费充能 +10%</t>
+          <t>装备效果等级 +15</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1865,16 +1865,16 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>free_charge</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H17" t="n">
-        <v>1</v>
+        <v>0.1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1882,17 +1882,17 @@
         </is>
       </c>
       <c r="J17" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>强化附加等级 +1</t>
+          <t>所有充能模块免费充能 +10%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B18" t="n">
         <v>3</v>
@@ -1917,11 +1917,11 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>equipment</t>
+          <t>enhancement</t>
         </is>
       </c>
       <c r="H18" t="n">
-        <v>15</v>
+        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1929,20 +1929,20 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>装备效果等级 +15</t>
+          <t>强化附加等级 +1</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B19" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1964,11 +1964,11 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>hightech</t>
+          <t>equipment</t>
         </is>
       </c>
       <c r="H19" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1976,20 +1976,20 @@
         </is>
       </c>
       <c r="J19" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>AI工厂效果等级 +10</t>
+          <t>装备效果等级 +15</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="B20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -2033,10 +2033,10 @@
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="B21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -2080,10 +2080,10 @@
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="B22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -2127,10 +2127,10 @@
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c r="B23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -2147,16 +2147,16 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>free_charge</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>hightech</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H23" t="n">
-        <v>10</v>
+        <v>0.1</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
@@ -2164,67 +2164,67 @@
         </is>
       </c>
       <c r="J23" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>AI工厂效果等级 +10</t>
+          <t>所有充能模块免费充能 +10%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B24" t="n">
+        <v>5</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>level_bonus</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>enhancement</t>
+        </is>
+      </c>
+      <c r="H24" t="n">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J24" t="n">
         <v>4</v>
       </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D24" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr">
-        <is>
-          <t>free_charge</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J24" t="n">
-        <v>3</v>
-      </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>所有充能模块免费充能 +10%</t>
+          <t>强化附加等级 +1</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="B25" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -2246,32 +2246,32 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>equipment</t>
         </is>
       </c>
       <c r="H25" t="n">
+        <v>15</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>add</t>
+        </is>
+      </c>
+      <c r="J25" t="n">
         <v>1</v>
       </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J25" t="n">
-        <v>4</v>
-      </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>强化附加等级 +1</t>
+          <t>装备效果等级 +15</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -2288,16 +2288,16 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>free_charge</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>equipment</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H26" t="n">
-        <v>15</v>
+        <v>0.1</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
@@ -2305,20 +2305,20 @@
         </is>
       </c>
       <c r="J26" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>装备效果等级 +15</t>
+          <t>所有充能模块免费充能 +10%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="B27" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -2340,11 +2340,11 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>hightech</t>
+          <t>enhancement</t>
         </is>
       </c>
       <c r="H27" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
@@ -2352,20 +2352,20 @@
         </is>
       </c>
       <c r="J27" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>AI工厂效果等级 +10</t>
+          <t>强化附加等级 +1</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="B28" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -2382,37 +2382,37 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>free_charge</t>
+          <t>planet_unlock</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>all</t>
+          <t>planet</t>
         </is>
       </c>
       <c r="H28" t="n">
-        <v>0.1</v>
+        <v>2</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>add</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J28" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>所有充能模块免费充能 +10%</t>
+          <t>能够探索新星球：气态巨星-T587e</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="B29" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -2429,178 +2429,178 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>planet_unlock</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>planet</t>
         </is>
       </c>
       <c r="H29" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>add</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J29" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>强化附加等级 +1</t>
+          <t>能够探索新星球：主序星-UTE334</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="B30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>planet_unlock</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>planet</t>
+        </is>
+      </c>
+      <c r="H30" t="n">
+        <v>4</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J30" t="n">
         <v>6</v>
       </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D30" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F30" t="inlineStr">
-        <is>
-          <t>level_bonus</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>equipment</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>15</v>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J30" t="n">
-        <v>1</v>
-      </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>装备效果等级 +15</t>
+          <t>能够探索新星球：红巨星-RG214</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>28</v>
+        <v>34</v>
       </c>
       <c r="B31" t="n">
+        <v>4</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>planet_unlock</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>planet</t>
+        </is>
+      </c>
+      <c r="H31" t="n">
+        <v>5</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>max</t>
+        </is>
+      </c>
+      <c r="J31" t="n">
         <v>6</v>
       </c>
-      <c r="C31" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D31" t="n">
-        <v>0</v>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>level_bonus</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>hightech</t>
-        </is>
-      </c>
-      <c r="H31" t="n">
-        <v>10</v>
-      </c>
-      <c r="I31" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J31" t="n">
-        <v>2</v>
-      </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>AI工厂效果等级 +10</t>
+          <t>能够探索新星球：白矮星-WS113</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="B32" t="n">
+        <v>5</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>conquer</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>conquered</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>planet_unlock</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>planet</t>
+        </is>
+      </c>
+      <c r="H32" t="n">
         <v>6</v>
       </c>
-      <c r="C32" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D32" t="n">
-        <v>0</v>
-      </c>
-      <c r="E32" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>free_charge</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>0.1</v>
-      </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>add</t>
+          <t>max</t>
         </is>
       </c>
       <c r="J32" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>所有充能模块免费充能 +10%</t>
+          <t>能够探索新星球：脉冲星-PSR T46+38</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="B33" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -2617,16 +2617,16 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>level_bonus</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>enhancement</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H33" t="n">
-        <v>1</v>
+        <v>100</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
@@ -2634,20 +2634,20 @@
         </is>
       </c>
       <c r="J33" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>强化附加等级 +1</t>
+          <t>永久幸运 +{value}</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>31</v>
+        <v>37</v>
       </c>
       <c r="B34" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -2664,37 +2664,37 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>planet_unlock</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>planet</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H34" t="n">
-        <v>2</v>
+        <v>100</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>add</t>
         </is>
       </c>
       <c r="J34" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>能够探索新星球：气态巨星-T587e</t>
+          <t>永久幸运 +{value}</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="B35" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -2711,37 +2711,37 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>planet_unlock</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>planet</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H35" t="n">
-        <v>3</v>
+        <v>100</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>add</t>
         </is>
       </c>
       <c r="J35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>能够探索新星球：主序星-UTE334</t>
+          <t>永久幸运 +{value}</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="B36" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -2758,37 +2758,37 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>planet_unlock</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>planet</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H36" t="n">
-        <v>4</v>
+        <v>100</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>add</t>
         </is>
       </c>
       <c r="J36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>能够探索新星球：红巨星-RG214</t>
+          <t>永久幸运 +{value}</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B37" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -2805,37 +2805,37 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>planet_unlock</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>planet</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H37" t="n">
-        <v>5</v>
+        <v>100</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>add</t>
         </is>
       </c>
       <c r="J37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>能够探索新星球：白矮星-WS113</t>
+          <t>永久幸运 +{value}</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>35</v>
+        <v>41</v>
       </c>
       <c r="B38" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -2852,308 +2852,26 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>planet_unlock</t>
+          <t>luck</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>planet</t>
+          <t>all</t>
         </is>
       </c>
       <c r="H38" t="n">
-        <v>6</v>
+        <v>100</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>max</t>
+          <t>add</t>
         </is>
       </c>
       <c r="J38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K38" t="inlineStr">
-        <is>
-          <t>能够探索新星球：脉冲星-PSR T46+38</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="n">
-        <v>36</v>
-      </c>
-      <c r="B39" t="n">
-        <v>1</v>
-      </c>
-      <c r="C39" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D39" t="n">
-        <v>0</v>
-      </c>
-      <c r="E39" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>100</v>
-      </c>
-      <c r="I39" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J39" t="n">
-        <v>7</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>永久幸运 +{value}</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="n">
-        <v>37</v>
-      </c>
-      <c r="B40" t="n">
-        <v>2</v>
-      </c>
-      <c r="C40" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D40" t="n">
-        <v>0</v>
-      </c>
-      <c r="E40" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H40" t="n">
-        <v>100</v>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>7</v>
-      </c>
-      <c r="K40" t="inlineStr">
-        <is>
-          <t>永久幸运 +{value}</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="n">
-        <v>38</v>
-      </c>
-      <c r="B41" t="n">
-        <v>3</v>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D41" t="n">
-        <v>0</v>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>100</v>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J41" t="n">
-        <v>7</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>永久幸运 +{value}</t>
-        </is>
-      </c>
-    </row>
-    <row r="42">
-      <c r="A42" t="n">
-        <v>39</v>
-      </c>
-      <c r="B42" t="n">
-        <v>4</v>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D42" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H42" t="n">
-        <v>100</v>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J42" t="n">
-        <v>7</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>永久幸运 +{value}</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="n">
-        <v>40</v>
-      </c>
-      <c r="B43" t="n">
-        <v>5</v>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>0</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>100</v>
-      </c>
-      <c r="I43" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J43" t="n">
-        <v>7</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>永久幸运 +{value}</t>
-        </is>
-      </c>
-    </row>
-    <row r="44">
-      <c r="A44" t="n">
-        <v>41</v>
-      </c>
-      <c r="B44" t="n">
-        <v>6</v>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>conquer</t>
-        </is>
-      </c>
-      <c r="D44" t="n">
-        <v>0</v>
-      </c>
-      <c r="E44" t="inlineStr">
-        <is>
-          <t>conquered</t>
-        </is>
-      </c>
-      <c r="F44" t="inlineStr">
-        <is>
-          <t>luck</t>
-        </is>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>all</t>
-        </is>
-      </c>
-      <c r="H44" t="n">
-        <v>100</v>
-      </c>
-      <c r="I44" t="inlineStr">
-        <is>
-          <t>add</t>
-        </is>
-      </c>
-      <c r="J44" t="n">
-        <v>7</v>
-      </c>
-      <c r="K44" t="inlineStr">
         <is>
           <t>永久幸运 +{value}</t>
         </is>

</xml_diff>